<commit_message>
Put the room reference before the name in the room subject
The subject is now entity:SSC_01-029_Shell-Space rather than
entity:SSC_Level-01_Shell-Space_01-029. The reference segment already
carries the level, so the separate level segment was repeating it; the
four SSC_Level-* entities the delivered ontology ships are untouched and
are still what the rooms hang off.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VjCgP8dvpZP7tmvN8uqvax
</commit_message>
<xml_diff>
--- a/projects/dar-cairo-room-naming/SSC_HQ_Room_Names.xlsx
+++ b/projects/dar-cairo-room-naming/SSC_HQ_Room_Names.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Chilled-Water_B-013</t>
+          <t>entity:SSC_B-013_Chilled-Water</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Vent-Plant_B-014</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Vent-Plant_B-014</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -789,7 +789,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Vent-Plant_B-008</t>
+          <t>entity:SSC_B-008_Vent-Plant</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -862,7 +862,7 @@
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Vent-Plant_B-014</t>
+          <t>entity:SSC_B-014_Vent-Plant</t>
         </is>
       </c>
       <c r="M6" s="2" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Sprinkler-And-Water_B-016</t>
+          <t>entity:SSC_B-016_Sprinkler-And-Water</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Main-Sec-Control-Room_B-025</t>
+          <t>entity:SSC_B-025_Main-Sec-Control-Room</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Corridor_B-030</t>
+          <t>entity:SSC_B-030_Corridor</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
@@ -1148,7 +1148,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_AV-Room_01-008</t>
+          <t>entity:SSC_01-008_AV-Room</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1216,7 +1216,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_IDF-1_01-027</t>
+          <t>entity:SSC_01-027_IDF-1</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_IDF-1_01-027</t>
+          <t>entity:SSC_01-027_IDF-1</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_IDF-2_01-039</t>
+          <t>entity:SSC_01-039_IDF-2</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1415,7 +1415,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_IDF-2_01-039</t>
+          <t>entity:SSC_01-039_IDF-2</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-029</t>
+          <t>entity:SSC_01-029_Shell-Space</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Corridor_01-013</t>
+          <t>entity:SSC_01-013_Corridor</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Printing_03-033</t>
+          <t>entity:SSC_03-033_Printing</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-B1_Entrance_B-015</t>
+          <t>entity:SSC_B-015_Entrance</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-014</t>
+          <t>entity:SSC_01-014_Shell-Space</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-014</t>
+          <t>entity:SSC_01-014_Shell-Space</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-014</t>
+          <t>entity:SSC_01-014_Shell-Space</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-015</t>
+          <t>entity:SSC_01-015_Shell-Space</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-015</t>
+          <t>entity:SSC_01-015_Shell-Space</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2128,7 +2128,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-015</t>
+          <t>entity:SSC_01-015_Shell-Space</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2201,7 +2201,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Corridor_01-024</t>
+          <t>entity:SSC_01-024_Corridor</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2274,7 +2274,7 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Corridor_01-001</t>
+          <t>entity:SSC_01-001_Corridor</t>
         </is>
       </c>
       <c r="M26" s="2" t="inlineStr">
@@ -2342,7 +2342,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Prayer-Room_01-019</t>
+          <t>entity:SSC_01-019_Prayer-Room</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Prayer-Room_01-019</t>
+          <t>entity:SSC_01-019_Prayer-Room</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2478,7 +2478,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Prayer-Room_01-019</t>
+          <t>entity:SSC_01-019_Prayer-Room</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2546,7 +2546,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Prayer-Room_01-019</t>
+          <t>entity:SSC_01-019_Prayer-Room</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Prayer-Room_01-019</t>
+          <t>entity:SSC_01-019_Prayer-Room</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Room-No-42_01-029</t>
+          <t>entity:SSC_01-029_Room-No-42</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Room-No-43_01-029</t>
+          <t>entity:SSC_01-029_Room-No-43</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2823,7 +2823,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Room-No-44_01-029</t>
+          <t>entity:SSC_01-029_Room-No-44</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2891,7 +2891,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-029</t>
+          <t>entity:SSC_01-029_Shell-Space</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2959,7 +2959,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-029</t>
+          <t>entity:SSC_01-029_Shell-Space</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -3027,7 +3027,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-029</t>
+          <t>entity:SSC_01-029_Shell-Space</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Corridor_01-013</t>
+          <t>entity:SSC_01-013_Corridor</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3173,7 +3173,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Open-Space_01-003</t>
+          <t>entity:SSC_01-003_Open-Space</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Open-Space_01-003</t>
+          <t>entity:SSC_01-003_Open-Space</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Open-Space_01-003</t>
+          <t>entity:SSC_01-003_Open-Space</t>
         </is>
       </c>
       <c r="M41" s="2" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-002</t>
+          <t>entity:SSC_01-002_Shell-Space</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3459,7 +3459,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-002</t>
+          <t>entity:SSC_01-002_Shell-Space</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3527,7 +3527,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-002</t>
+          <t>entity:SSC_01-002_Shell-Space</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-002</t>
+          <t>entity:SSC_01-002_Shell-Space</t>
         </is>
       </c>
       <c r="M45" s="2" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Open-Space_01-003</t>
+          <t>entity:SSC_01-003_Open-Space</t>
         </is>
       </c>
       <c r="M46" s="2" t="inlineStr">
@@ -3750,7 +3750,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Shell-Space_01-016</t>
+          <t>entity:SSC_01-016_Shell-Space</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3823,7 +3823,7 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Open-Space_01-003</t>
+          <t>entity:SSC_01-003_Open-Space</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
@@ -3896,7 +3896,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Corridor_01-018</t>
+          <t>entity:SSC_01-018_Corridor</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3973,7 +3973,7 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_IDF-2_01-039</t>
+          <t>entity:SSC_01-039_IDF-2</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
@@ -4050,7 +4050,7 @@
       </c>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Open-Space_01-003</t>
+          <t>entity:SSC_01-003_Open-Space</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
@@ -4127,7 +4127,7 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Corridor_01-028</t>
+          <t>entity:SSC_01-028_Corridor</t>
         </is>
       </c>
       <c r="M52" s="2" t="inlineStr">
@@ -4204,7 +4204,7 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Prayer-Room_01-019</t>
+          <t>entity:SSC_01-019_Prayer-Room</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr">
@@ -4272,7 +4272,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_AV-Room_01-008</t>
+          <t>entity:SSC_01-008_AV-Room</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Stair-4_01-ST-4</t>
+          <t>entity:SSC_01-ST-4_Stair-4</t>
         </is>
       </c>
       <c r="M55" s="2" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-01_Open-Space_01-003</t>
+          <t>entity:SSC_01-003_Open-Space</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr">
@@ -4494,7 +4494,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Conference-Room_02-006</t>
+          <t>entity:SSC_02-006_Conference-Room</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -4562,7 +4562,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Executive-Conference-Room_02-005</t>
+          <t>entity:SSC_02-005_Executive-Conference-Room</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Executive-Conference-Room_02-005</t>
+          <t>entity:SSC_02-005_Executive-Conference-Room</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Corridor_02-004</t>
+          <t>entity:SSC_02-004_Corridor</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Foyer_02-001</t>
+          <t>entity:SSC_02-001_Foyer</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Foyer_02-001</t>
+          <t>entity:SSC_02-001_Foyer</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -4887,7 +4887,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Lobby_02-002</t>
+          <t>entity:SSC_02-002_Lobby</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -4955,7 +4955,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Lobby_02-002</t>
+          <t>entity:SSC_02-002_Lobby</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -5023,7 +5023,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Lobby_02-002</t>
+          <t>entity:SSC_02-002_Lobby</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -5096,7 +5096,7 @@
       </c>
       <c r="L66" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Corridor_02-003</t>
+          <t>entity:SSC_02-003_Corridor</t>
         </is>
       </c>
       <c r="M66" s="2" t="inlineStr">
@@ -5169,7 +5169,7 @@
       </c>
       <c r="L67" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Lobby_02-002</t>
+          <t>entity:SSC_02-002_Lobby</t>
         </is>
       </c>
       <c r="M67" s="2" t="inlineStr">
@@ -5237,7 +5237,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Executive-Conference-Room_02-005</t>
+          <t>entity:SSC_02-005_Executive-Conference-Room</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -5305,7 +5305,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-02_Conference-Room_02-006</t>
+          <t>entity:SSC_02-006_Conference-Room</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -5373,7 +5373,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-015</t>
+          <t>entity:SSC_03-015_Researchers-Office</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Visitors-Cubicle_03-014</t>
+          <t>entity:SSC_03-014_Visitors-Cubicle</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -5509,7 +5509,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-013</t>
+          <t>entity:SSC_03-013_Researchers-Office</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -5577,7 +5577,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-012</t>
+          <t>entity:SSC_03-012_Researchers-Office</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -5645,7 +5645,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Visitors-Cubicle_03-011</t>
+          <t>entity:SSC_03-011_Visitors-Cubicle</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -5713,7 +5713,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-010</t>
+          <t>entity:SSC_03-010_Researchers-Office</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -5781,7 +5781,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-009</t>
+          <t>entity:SSC_03-009_Researchers-Office</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -5849,7 +5849,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Visitors-Cubicle_03-008</t>
+          <t>entity:SSC_03-008_Visitors-Cubicle</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -5917,7 +5917,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Operations-Manager_03-007</t>
+          <t>entity:SSC_03-007_Operations-Manager</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -5990,7 +5990,7 @@
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Room_03-006A</t>
+          <t>entity:SSC_03-006A_Room</t>
         </is>
       </c>
       <c r="M79" s="2" t="inlineStr">
@@ -6098,7 +6098,7 @@
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Room_03-006B</t>
+          <t>entity:SSC_03-006B_Room</t>
         </is>
       </c>
       <c r="M81" s="2" t="inlineStr">
@@ -6161,7 +6161,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-005</t>
+          <t>entity:SSC_03-005_Researchers-Office</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Visitors-Cubicle_03-004</t>
+          <t>entity:SSC_03-004_Visitors-Cubicle</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-003</t>
+          <t>entity:SSC_03-003_Researchers-Office</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -6350,7 +6350,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Directors-Meeting-Room_03-002</t>
+          <t>entity:SSC_03-002_Directors-Meeting-Room</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -6413,7 +6413,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Directors-Meeting-Room_03-002</t>
+          <t>entity:SSC_03-002_Directors-Meeting-Room</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -6476,7 +6476,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Directors-Office_03-001</t>
+          <t>entity:SSC_03-001_Directors-Office</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -6549,7 +6549,7 @@
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_General-Office-Area_03-032</t>
+          <t>entity:SSC_03-032_General-Office-Area</t>
         </is>
       </c>
       <c r="M88" s="2" t="inlineStr">
@@ -6622,7 +6622,7 @@
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_General-Office-Area_03-032</t>
+          <t>entity:SSC_03-032_General-Office-Area</t>
         </is>
       </c>
       <c r="M89" s="2" t="inlineStr">
@@ -6695,7 +6695,7 @@
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_General-Office-Area_03-032</t>
+          <t>entity:SSC_03-032_General-Office-Area</t>
         </is>
       </c>
       <c r="M90" s="2" t="inlineStr">
@@ -6768,7 +6768,7 @@
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_General-Office-Area_03-032</t>
+          <t>entity:SSC_03-032_General-Office-Area</t>
         </is>
       </c>
       <c r="M91" s="2" t="inlineStr">
@@ -6841,7 +6841,7 @@
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_General-Office-Area_03-032</t>
+          <t>entity:SSC_03-032_General-Office-Area</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr">
@@ -6914,7 +6914,7 @@
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Assoc-Directors-Office_03-031</t>
+          <t>entity:SSC_03-031_Assoc-Directors-Office</t>
         </is>
       </c>
       <c r="M93" s="2" t="inlineStr">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_General-Office-Area_03-032</t>
+          <t>entity:SSC_03-032_General-Office-Area</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr">
@@ -7055,7 +7055,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Assoc-Directors-Office_03-031</t>
+          <t>entity:SSC_03-031_Assoc-Directors-Office</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -7118,7 +7118,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Assoc-Directors-Meeting-Room_03-030</t>
+          <t>entity:SSC_03-030_Assoc-Directors-Meeting-Room</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -7186,7 +7186,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Assoc-Directors-Meeting-Room_03-030</t>
+          <t>entity:SSC_03-030_Assoc-Directors-Meeting-Room</t>
         </is>
       </c>
       <c r="M97" t="inlineStr">
@@ -7254,7 +7254,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-029</t>
+          <t>entity:SSC_03-029_Researchers-Office</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -7322,7 +7322,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Visitors-Cubicle_03-028</t>
+          <t>entity:SSC_03-028_Visitors-Cubicle</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
@@ -7390,7 +7390,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-027</t>
+          <t>entity:SSC_03-027_Researchers-Office</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
@@ -7458,7 +7458,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Meeting-Room_03-026</t>
+          <t>entity:SSC_03-026_Meeting-Room</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
@@ -7526,7 +7526,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Meeting-Room_03-026</t>
+          <t>entity:SSC_03-026_Meeting-Room</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -7594,7 +7594,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Meeting-Room_03-026</t>
+          <t>entity:SSC_03-026_Meeting-Room</t>
         </is>
       </c>
       <c r="M103" t="inlineStr">
@@ -7662,7 +7662,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Secretarial-Area_03-025</t>
+          <t>entity:SSC_03-025_Secretarial-Area</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Visitors-Cubicle_03-024</t>
+          <t>entity:SSC_03-024_Visitors-Cubicle</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
@@ -7798,7 +7798,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-023</t>
+          <t>entity:SSC_03-023_Researchers-Office</t>
         </is>
       </c>
       <c r="M106" t="inlineStr">
@@ -7866,7 +7866,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-022</t>
+          <t>entity:SSC_03-022_Researchers-Office</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Visitors-Cubicle_03-021</t>
+          <t>entity:SSC_03-021_Visitors-Cubicle</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -8002,7 +8002,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-020</t>
+          <t>entity:SSC_03-020_Researchers-Office</t>
         </is>
       </c>
       <c r="M109" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_IT-Managers-Office_03-019</t>
+          <t>entity:SSC_03-019_IT-Managers-Office</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
@@ -8138,7 +8138,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Visitors-Cubicle_03-018</t>
+          <t>entity:SSC_03-018_Visitors-Cubicle</t>
         </is>
       </c>
       <c r="M111" t="inlineStr">
@@ -8206,7 +8206,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Researchers-Office_03-017</t>
+          <t>entity:SSC_03-017_Researchers-Office</t>
         </is>
       </c>
       <c r="M112" t="inlineStr">
@@ -8274,7 +8274,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Lounge_03-016</t>
+          <t>entity:SSC_03-016_Lounge</t>
         </is>
       </c>
       <c r="M113" t="inlineStr">
@@ -8342,7 +8342,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Lounge_03-016</t>
+          <t>entity:SSC_03-016_Lounge</t>
         </is>
       </c>
       <c r="M114" t="inlineStr">
@@ -8415,7 +8415,7 @@
       </c>
       <c r="L115" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Lounge_03-016</t>
+          <t>entity:SSC_03-016_Lounge</t>
         </is>
       </c>
       <c r="M115" s="2" t="inlineStr">
@@ -8488,7 +8488,7 @@
       </c>
       <c r="L116" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Corridor_03-034</t>
+          <t>entity:SSC_03-034_Corridor</t>
         </is>
       </c>
       <c r="M116" s="2" t="inlineStr">
@@ -8551,7 +8551,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Corridor_03-041</t>
+          <t>entity:SSC_03-041_Corridor</t>
         </is>
       </c>
       <c r="M117" t="inlineStr">
@@ -8624,7 +8624,7 @@
       </c>
       <c r="L118" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Corridor_03-042</t>
+          <t>entity:SSC_03-042_Corridor</t>
         </is>
       </c>
       <c r="M118" s="2" t="inlineStr">
@@ -8701,7 +8701,7 @@
       </c>
       <c r="L119" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Corridor_03-041</t>
+          <t>entity:SSC_03-041_Corridor</t>
         </is>
       </c>
       <c r="M119" s="2" t="inlineStr">
@@ -8769,7 +8769,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Corridor_03-034</t>
+          <t>entity:SSC_03-034_Corridor</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
@@ -8837,7 +8837,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Corridor_03-034</t>
+          <t>entity:SSC_03-034_Corridor</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
@@ -8905,7 +8905,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Corridor_03-034</t>
+          <t>entity:SSC_03-034_Corridor</t>
         </is>
       </c>
       <c r="M122" t="inlineStr">
@@ -8973,7 +8973,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_Corridor_03-042</t>
+          <t>entity:SSC_03-042_Corridor</t>
         </is>
       </c>
       <c r="M123" t="inlineStr">
@@ -9050,7 +9050,7 @@
       </c>
       <c r="L124" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_General-Office-Area_03-032</t>
+          <t>entity:SSC_03-032_General-Office-Area</t>
         </is>
       </c>
       <c r="M124" s="2" t="inlineStr">
@@ -9127,7 +9127,7 @@
       </c>
       <c r="L125" s="2" t="inlineStr">
         <is>
-          <t>entity:SSC_Level-03_General-Office-Area_03-032</t>
+          <t>entity:SSC_03-032_General-Office-Area</t>
         </is>
       </c>
       <c r="M125" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Take the 3F-Roof reading for VAV0092-93
Level 1 belongs to the B-2F split, but 3F-Roof's own column H and the
delivered HQ draft both put the finance cashier in 1.106 and the secure
room in 1.116. The client read the three flagged conflicts and chose
3F-Roof for this pair and B-2F for VAV0039-41, VAV0052-53 and VAV0090,
which is what the level rule already gave.

The exception is a named table rather than an edited cell, and both rows
carry the reason in their notes. The sheet and the HQ draft now agree on
these two rooms.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VjCgP8dvpZP7tmvN8uqvax
</commit_message>
<xml_diff>
--- a/projects/dar-cairo-room-naming/SSC_HQ_Room_Names.xlsx
+++ b/projects/dar-cairo-room-naming/SSC_HQ_Room_Names.xlsx
@@ -26263,12 +26263,12 @@
       </c>
       <c r="D250" s="2" t="inlineStr">
         <is>
-          <t>FINANCE CASHIER 1.116</t>
+          <t>FINANCE CASHIER 1.106</t>
         </is>
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>entity:HQ_1.116_FINANCE_CASHIER</t>
+          <t>entity:HQ_1.106_FINANCE_CASHIER</t>
         </is>
       </c>
       <c r="F250" s="2" t="n"/>
@@ -26281,7 +26281,7 @@
       </c>
       <c r="J250" s="2" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>106</t>
         </is>
       </c>
       <c r="K250" s="2" t="inlineStr">
@@ -26291,12 +26291,12 @@
       </c>
       <c r="L250" s="2" t="inlineStr">
         <is>
-          <t>entity:HQ_1-116_Finance-Cashier</t>
+          <t>entity:HQ_1-106_Finance-Cashier</t>
         </is>
       </c>
       <c r="M250" s="2" t="inlineStr">
         <is>
-          <t>1.116 FINANCE CASHIER</t>
+          <t>1.106 FINANCE CASHIER</t>
         </is>
       </c>
       <c r="N250" s="2" t="inlineStr">
@@ -26306,7 +26306,7 @@
       </c>
       <c r="O250" s="2" t="inlineStr">
         <is>
-          <t>D disagrees between the two workbooks - sources/HQ_rooms_B-2F.xlsx says 'FINANCE CASHIER 1.116', sources/HQ_rooms_3F-Roof.xlsx says 'FINANCE CASHIER 1.106'; sources/HQ_rooms_B-2F.xlsx owns this level; E disagrees between the two workbooks - sources/HQ_rooms_B-2F.xlsx says 'entity:HQ_1.116_FINANCE_CASHIER', sources/HQ_rooms_3F-Roof.xlsx says 'entity:HQ_1.106_FINANCE_CASHIER'; sources/HQ_rooms_B-2F.xlsx owns this level; no usable J, so column D stands; QF_HQ_Ontology_draft0.4.xlsx calls 1.116 'FINANCE SECURE ROOM'</t>
+          <t>the level rule points at the other workbook here; sources/HQ_rooms_3F-Roof.xlsx was chosen for this row on the client's instruction; D disagrees between the two workbooks - sources/HQ_rooms_3F-Roof.xlsx says 'FINANCE CASHIER 1.106', sources/HQ_rooms_B-2F.xlsx says 'FINANCE CASHIER 1.116'; sources/HQ_rooms_3F-Roof.xlsx owns this level; E disagrees between the two workbooks - sources/HQ_rooms_3F-Roof.xlsx says 'entity:HQ_1.106_FINANCE_CASHIER', sources/HQ_rooms_B-2F.xlsx says 'entity:HQ_1.116_FINANCE_CASHIER'; sources/HQ_rooms_3F-Roof.xlsx owns this level; no usable J, so column D stands</t>
         </is>
       </c>
     </row>
@@ -26328,12 +26328,12 @@
       </c>
       <c r="D251" s="2" t="inlineStr">
         <is>
-          <t>FINANCE ROOM 1.106</t>
+          <t>FINANCE ROOM 1.116</t>
         </is>
       </c>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>entity:HQ_1.106_FINANCE_SECURE_ROOM</t>
+          <t>entity:HQ_1.116_FINANCE_SECURE_ROOM</t>
         </is>
       </c>
       <c r="F251" s="2" t="inlineStr">
@@ -26341,11 +26341,7 @@
           <t>FINANCE SECURE ROOM 1.116</t>
         </is>
       </c>
-      <c r="G251" s="2" t="inlineStr">
-        <is>
-          <t>1.106 FINANCE ROOM</t>
-        </is>
-      </c>
+      <c r="G251" s="2" t="n"/>
       <c r="H251" s="2" t="inlineStr"/>
       <c r="I251" s="2" t="inlineStr">
         <is>
@@ -26354,7 +26350,7 @@
       </c>
       <c r="J251" s="2" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>116</t>
         </is>
       </c>
       <c r="K251" s="2" t="inlineStr">
@@ -26364,12 +26360,12 @@
       </c>
       <c r="L251" s="2" t="inlineStr">
         <is>
-          <t>entity:HQ_1-106_Finance-Secure-Room</t>
+          <t>entity:HQ_1-116_Finance-Secure-Room</t>
         </is>
       </c>
       <c r="M251" s="2" t="inlineStr">
         <is>
-          <t>1.106 FINANCE SECURE ROOM</t>
+          <t>1.116 FINANCE SECURE ROOM</t>
         </is>
       </c>
       <c r="N251" s="2" t="inlineStr">
@@ -26379,7 +26375,7 @@
       </c>
       <c r="O251" s="2" t="inlineStr">
         <is>
-          <t>D disagrees between the two workbooks - sources/HQ_rooms_B-2F.xlsx says 'FINANCE ROOM 1.106', sources/HQ_rooms_3F-Roof.xlsx says 'FINANCE ROOM 1.116'; sources/HQ_rooms_B-2F.xlsx owns this level; E disagrees between the two workbooks - sources/HQ_rooms_B-2F.xlsx says 'entity:HQ_1.106_FINANCE_SECURE_ROOM', sources/HQ_rooms_3F-Roof.xlsx says 'entity:HQ_1.116_FINANCE_SECURE_ROOM'; sources/HQ_rooms_B-2F.xlsx owns this level; column H was blank in sources/HQ_rooms_B-2F.xlsx, taken from sources/HQ_rooms_3F-Roof.xlsx; H carries a room number, so column D stands; D (FINANCE ROOM) does not match E - name taken from E; QF_HQ_Ontology_draft0.4.xlsx calls 1.106 'FINANCE CASHIER'</t>
+          <t>the level rule points at the other workbook here; sources/HQ_rooms_3F-Roof.xlsx was chosen for this row on the client's instruction; D disagrees between the two workbooks - sources/HQ_rooms_3F-Roof.xlsx says 'FINANCE ROOM 1.116', sources/HQ_rooms_B-2F.xlsx says 'FINANCE ROOM 1.106'; sources/HQ_rooms_3F-Roof.xlsx owns this level; E disagrees between the two workbooks - sources/HQ_rooms_3F-Roof.xlsx says 'entity:HQ_1.116_FINANCE_SECURE_ROOM', sources/HQ_rooms_B-2F.xlsx says 'entity:HQ_1.106_FINANCE_SECURE_ROOM'; sources/HQ_rooms_3F-Roof.xlsx owns this level; H carries a room number, so column D stands; D (FINANCE ROOM) does not match E - name taken from E</t>
         </is>
       </c>
     </row>

</xml_diff>